<commit_message>
Updated audiomoth metadata again.
</commit_message>
<xml_diff>
--- a/audiomoth_data/audiomoth_metadata.xlsx
+++ b/audiomoth_data/audiomoth_metadata.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\charl\Documents\University\Year 5 Masters\Research Project\2. Analysis\final_research_project\audiomoth_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D32A079-5C99-4B1F-B635-11310594030B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{835684E4-1A3B-40ED-8963-70ADEFDF6842}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="609" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="717" uniqueCount="40">
   <si>
     <t>site</t>
   </si>
@@ -131,6 +131,15 @@
   </si>
   <si>
     <t>SanDiskExtreme</t>
+  </si>
+  <si>
+    <t>case_checked</t>
+  </si>
+  <si>
+    <t>Y</t>
+  </si>
+  <si>
+    <t>EB</t>
   </si>
 </sst>
 </file>
@@ -492,16 +501,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I121"/>
+  <dimension ref="A1:J129"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="20.6640625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="22.109375" style="2" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="13.77734375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="10.5546875" style="4" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="10.21875" style="4" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.6640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:10" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -529,8 +539,11 @@
       <c r="I1" s="3" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J1" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>7</v>
       </c>
@@ -559,7 +572,7 @@
         <v>-3.4026420000000002</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>7</v>
       </c>
@@ -588,7 +601,7 @@
         <v>-3.4026420000000002</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>7</v>
       </c>
@@ -617,7 +630,7 @@
         <v>-3.4026420000000002</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>7</v>
       </c>
@@ -645,8 +658,11 @@
       <c r="I5" s="4">
         <v>-3.4047040000000002</v>
       </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J5" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>7</v>
       </c>
@@ -674,8 +690,11 @@
       <c r="I6" s="4">
         <v>-3.4047040000000002</v>
       </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J6" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>7</v>
       </c>
@@ -703,8 +722,11 @@
       <c r="I7" s="4">
         <v>-3.4047040000000002</v>
       </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J7" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>7</v>
       </c>
@@ -733,7 +755,7 @@
         <v>-3.4009160000000001</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>7</v>
       </c>
@@ -762,7 +784,7 @@
         <v>-3.4009160000000001</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>7</v>
       </c>
@@ -791,7 +813,7 @@
         <v>-3.4009160000000001</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>7</v>
       </c>
@@ -819,8 +841,11 @@
       <c r="I11" s="4">
         <v>-3.4025940000000001</v>
       </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J11" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>7</v>
       </c>
@@ -848,8 +873,11 @@
       <c r="I12" s="4">
         <v>-3.4025940000000001</v>
       </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J12" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>7</v>
       </c>
@@ -877,8 +905,11 @@
       <c r="I13" s="4">
         <v>-3.4025940000000001</v>
       </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J13" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
         <v>7</v>
       </c>
@@ -907,7 +938,7 @@
         <v>-3.4005800000000002</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>7</v>
       </c>
@@ -936,7 +967,7 @@
         <v>-3.4005800000000002</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>7</v>
       </c>
@@ -965,7 +996,7 @@
         <v>-3.4005800000000002</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
         <v>7</v>
       </c>
@@ -994,7 +1025,7 @@
         <v>-3.403073</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
         <v>7</v>
       </c>
@@ -1023,7 +1054,7 @@
         <v>-3.403073</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
         <v>7</v>
       </c>
@@ -1052,7 +1083,7 @@
         <v>-3.403073</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
         <v>7</v>
       </c>
@@ -1081,7 +1112,7 @@
         <v>-3.401923</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
         <v>7</v>
       </c>
@@ -1110,7 +1141,7 @@
         <v>-3.401923</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
         <v>7</v>
       </c>
@@ -1139,7 +1170,7 @@
         <v>-3.401923</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
         <v>7</v>
       </c>
@@ -1167,8 +1198,11 @@
       <c r="I23" s="4">
         <v>-3.4018269999999999</v>
       </c>
-    </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J23" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
         <v>7</v>
       </c>
@@ -1196,8 +1230,11 @@
       <c r="I24" s="4">
         <v>-3.4018269999999999</v>
       </c>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J24" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
         <v>7</v>
       </c>
@@ -1225,8 +1262,11 @@
       <c r="I25" s="4">
         <v>-3.4018269999999999</v>
       </c>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J25" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
         <v>7</v>
       </c>
@@ -1254,8 +1294,11 @@
       <c r="I26" s="4">
         <v>-3.4039839999999999</v>
       </c>
-    </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J26" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
         <v>7</v>
       </c>
@@ -1283,8 +1326,11 @@
       <c r="I27" s="4">
         <v>-3.4039839999999999</v>
       </c>
-    </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J27" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
         <v>7</v>
       </c>
@@ -1312,8 +1358,11 @@
       <c r="I28" s="4">
         <v>-3.4039839999999999</v>
       </c>
-    </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J28" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
         <v>7</v>
       </c>
@@ -1341,8 +1390,11 @@
       <c r="I29" s="4">
         <v>-3.4024019999999999</v>
       </c>
-    </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J29" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="30" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
         <v>7</v>
       </c>
@@ -1370,8 +1422,11 @@
       <c r="I30" s="4">
         <v>-3.4024019999999999</v>
       </c>
-    </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J30" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
         <v>7</v>
       </c>
@@ -1399,8 +1454,11 @@
       <c r="I31" s="4">
         <v>-3.4024019999999999</v>
       </c>
-    </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J31" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
         <v>7</v>
       </c>
@@ -1429,7 +1487,7 @@
         <v>-3.4025940000000001</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
         <v>7</v>
       </c>
@@ -1458,7 +1516,7 @@
         <v>-3.4025940000000001</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
         <v>7</v>
       </c>
@@ -1487,7 +1545,7 @@
         <v>-3.4025940000000001</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
         <v>7</v>
       </c>
@@ -1515,8 +1573,11 @@
       <c r="I35" s="4">
         <v>-3.4033129999999998</v>
       </c>
-    </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J35" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
         <v>7</v>
       </c>
@@ -1544,8 +1605,11 @@
       <c r="I36" s="4">
         <v>-3.4033129999999998</v>
       </c>
-    </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J36" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
         <v>7</v>
       </c>
@@ -1573,8 +1637,11 @@
       <c r="I37" s="4">
         <v>-3.4033129999999998</v>
       </c>
-    </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J37" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
         <v>7</v>
       </c>
@@ -1602,8 +1669,11 @@
       <c r="I38" s="4">
         <v>-3.4039839999999999</v>
       </c>
-    </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J38" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
         <v>7</v>
       </c>
@@ -1631,8 +1701,11 @@
       <c r="I39" s="4">
         <v>-3.4039839999999999</v>
       </c>
-    </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J39" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
         <v>7</v>
       </c>
@@ -1660,8 +1733,11 @@
       <c r="I40" s="4">
         <v>-3.4039839999999999</v>
       </c>
-    </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J40" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
         <v>7</v>
       </c>
@@ -1690,7 +1766,7 @@
         <v>-3.4015390000000001</v>
       </c>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
         <v>7</v>
       </c>
@@ -1719,7 +1795,7 @@
         <v>-3.4015390000000001</v>
       </c>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
         <v>7</v>
       </c>
@@ -1748,7 +1824,7 @@
         <v>-3.4015390000000001</v>
       </c>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
         <v>7</v>
       </c>
@@ -1776,8 +1852,11 @@
       <c r="I44" s="4">
         <v>-3.4033609999999999</v>
       </c>
-    </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J44" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
         <v>7</v>
       </c>
@@ -1805,8 +1884,11 @@
       <c r="I45" s="4">
         <v>-3.4033609999999999</v>
       </c>
-    </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J45" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
         <v>7</v>
       </c>
@@ -1834,8 +1916,11 @@
       <c r="I46" s="4">
         <v>-3.4033609999999999</v>
       </c>
-    </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J46" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
         <v>7</v>
       </c>
@@ -1863,8 +1948,11 @@
       <c r="I47" s="4">
         <v>-3.400388</v>
       </c>
-    </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J47" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
         <v>7</v>
       </c>
@@ -1892,8 +1980,11 @@
       <c r="I48" s="4">
         <v>-3.400388</v>
       </c>
-    </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J48" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="49" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
         <v>7</v>
       </c>
@@ -1921,8 +2012,11 @@
       <c r="I49" s="4">
         <v>-3.400388</v>
       </c>
-    </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J49" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="50" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
         <v>7</v>
       </c>
@@ -1950,8 +2044,11 @@
       <c r="I50" s="4">
         <v>-3.403019</v>
       </c>
-    </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J50" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="51" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
         <v>7</v>
       </c>
@@ -1979,8 +2076,11 @@
       <c r="I51" s="4">
         <v>-3.403019</v>
       </c>
-    </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J51" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="52" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
         <v>7</v>
       </c>
@@ -2008,8 +2108,11 @@
       <c r="I52" s="4">
         <v>-3.403019</v>
       </c>
-    </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J52" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="53" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
         <v>7</v>
       </c>
@@ -2037,8 +2140,11 @@
       <c r="I53" s="4">
         <v>-3.3997649999999999</v>
       </c>
-    </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J53" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="54" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
         <v>7</v>
       </c>
@@ -2066,8 +2172,11 @@
       <c r="I54" s="4">
         <v>-3.3997649999999999</v>
       </c>
-    </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J54" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="55" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
         <v>7</v>
       </c>
@@ -2095,8 +2204,11 @@
       <c r="I55" s="4">
         <v>-3.3997649999999999</v>
       </c>
-    </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J55" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="56" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A56" t="s">
         <v>7</v>
       </c>
@@ -2124,8 +2236,11 @@
       <c r="I56" s="4">
         <v>-3.401443</v>
       </c>
-    </row>
-    <row r="57" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J56" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="57" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
         <v>7</v>
       </c>
@@ -2153,8 +2268,11 @@
       <c r="I57" s="4">
         <v>-3.401443</v>
       </c>
-    </row>
-    <row r="58" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J57" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="58" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A58" t="s">
         <v>7</v>
       </c>
@@ -2182,8 +2300,11 @@
       <c r="I58" s="4">
         <v>-3.401443</v>
       </c>
-    </row>
-    <row r="59" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J58" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="59" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A59" t="s">
         <v>7</v>
       </c>
@@ -2211,8 +2332,11 @@
       <c r="I59" s="4">
         <v>-3.4011559999999998</v>
       </c>
-    </row>
-    <row r="60" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J59" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="60" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A60" t="s">
         <v>7</v>
       </c>
@@ -2240,8 +2364,11 @@
       <c r="I60" s="4">
         <v>-3.4011559999999998</v>
       </c>
-    </row>
-    <row r="61" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J60" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="61" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
         <v>7</v>
       </c>
@@ -2269,8 +2396,11 @@
       <c r="I61" s="4">
         <v>-3.4011559999999998</v>
       </c>
-    </row>
-    <row r="62" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J61" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="62" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
         <v>29</v>
       </c>
@@ -2299,7 +2429,7 @@
         <v>-3.4046675999999998</v>
       </c>
     </row>
-    <row r="63" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A63" t="s">
         <v>29</v>
       </c>
@@ -2328,7 +2458,7 @@
         <v>-3.4046675999999998</v>
       </c>
     </row>
-    <row r="64" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A64" t="s">
         <v>29</v>
       </c>
@@ -2357,7 +2487,7 @@
         <v>-3.4046675999999998</v>
       </c>
     </row>
-    <row r="65" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
         <v>29</v>
       </c>
@@ -2385,8 +2515,11 @@
       <c r="I65" s="4">
         <v>-3.4032567999999999</v>
       </c>
-    </row>
-    <row r="66" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J65" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="66" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A66" t="s">
         <v>29</v>
       </c>
@@ -2414,8 +2547,11 @@
       <c r="I66" s="4">
         <v>-3.4032567999999999</v>
       </c>
-    </row>
-    <row r="67" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J66" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="67" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A67" t="s">
         <v>29</v>
       </c>
@@ -2443,8 +2579,11 @@
       <c r="I67" s="4">
         <v>-3.4032567999999999</v>
       </c>
-    </row>
-    <row r="68" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J67" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="68" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A68" t="s">
         <v>29</v>
       </c>
@@ -2473,7 +2612,7 @@
         <v>-3.4023837000000001</v>
       </c>
     </row>
-    <row r="69" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A69" t="s">
         <v>29</v>
       </c>
@@ -2502,7 +2641,7 @@
         <v>-3.4023837000000001</v>
       </c>
     </row>
-    <row r="70" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A70" t="s">
         <v>29</v>
       </c>
@@ -2531,7 +2670,7 @@
         <v>-3.4023837000000001</v>
       </c>
     </row>
-    <row r="71" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A71" t="s">
         <v>29</v>
       </c>
@@ -2559,8 +2698,11 @@
       <c r="I71" s="4">
         <v>-3.4053393999999999</v>
       </c>
-    </row>
-    <row r="72" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J71" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="72" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A72" t="s">
         <v>29</v>
       </c>
@@ -2588,8 +2730,11 @@
       <c r="I72" s="4">
         <v>-3.4053393999999999</v>
       </c>
-    </row>
-    <row r="73" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J72" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="73" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A73" t="s">
         <v>29</v>
       </c>
@@ -2617,8 +2762,11 @@
       <c r="I73" s="4">
         <v>-3.4053393999999999</v>
       </c>
-    </row>
-    <row r="74" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J73" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="74" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A74" t="s">
         <v>29</v>
       </c>
@@ -2647,7 +2795,7 @@
         <v>-3.4048367000000002</v>
       </c>
     </row>
-    <row r="75" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A75" t="s">
         <v>29</v>
       </c>
@@ -2676,7 +2824,7 @@
         <v>-3.4048367000000002</v>
       </c>
     </row>
-    <row r="76" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A76" t="s">
         <v>29</v>
       </c>
@@ -2705,7 +2853,7 @@
         <v>-3.4048367000000002</v>
       </c>
     </row>
-    <row r="77" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A77" t="s">
         <v>29</v>
       </c>
@@ -2734,7 +2882,7 @@
         <v>-3.4052387</v>
       </c>
     </row>
-    <row r="78" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A78" t="s">
         <v>29</v>
       </c>
@@ -2763,7 +2911,7 @@
         <v>-3.4052387</v>
       </c>
     </row>
-    <row r="79" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A79" t="s">
         <v>29</v>
       </c>
@@ -2792,7 +2940,7 @@
         <v>-3.4052387</v>
       </c>
     </row>
-    <row r="80" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A80" t="s">
         <v>29</v>
       </c>
@@ -2821,7 +2969,7 @@
         <v>-3.4047087</v>
       </c>
     </row>
-    <row r="81" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A81" t="s">
         <v>29</v>
       </c>
@@ -2850,7 +2998,7 @@
         <v>-3.4047087</v>
       </c>
     </row>
-    <row r="82" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A82" t="s">
         <v>29</v>
       </c>
@@ -2879,7 +3027,7 @@
         <v>-3.4047087</v>
       </c>
     </row>
-    <row r="83" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A83" t="s">
         <v>29</v>
       </c>
@@ -2907,8 +3055,11 @@
       <c r="I83" s="4">
         <v>-3.4029975000000001</v>
       </c>
-    </row>
-    <row r="84" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J83" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="84" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A84" t="s">
         <v>29</v>
       </c>
@@ -2936,8 +3087,11 @@
       <c r="I84" s="4">
         <v>-3.4029975000000001</v>
       </c>
-    </row>
-    <row r="85" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J84" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="85" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A85" t="s">
         <v>29</v>
       </c>
@@ -2965,8 +3119,11 @@
       <c r="I85" s="4">
         <v>-3.4029975000000001</v>
       </c>
-    </row>
-    <row r="86" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J85" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="86" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A86" t="s">
         <v>29</v>
       </c>
@@ -2994,8 +3151,11 @@
       <c r="I86" s="4">
         <v>-3.4028046000000001</v>
       </c>
-    </row>
-    <row r="87" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J86" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="87" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A87" t="s">
         <v>29</v>
       </c>
@@ -3023,8 +3183,11 @@
       <c r="I87" s="4">
         <v>-3.4028046000000001</v>
       </c>
-    </row>
-    <row r="88" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J87" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="88" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A88" t="s">
         <v>29</v>
       </c>
@@ -3052,8 +3215,11 @@
       <c r="I88" s="4">
         <v>-3.4028046000000001</v>
       </c>
-    </row>
-    <row r="89" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J88" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="89" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A89" t="s">
         <v>29</v>
       </c>
@@ -3081,8 +3247,11 @@
       <c r="I89" s="4">
         <v>-3.4041242999999999</v>
       </c>
-    </row>
-    <row r="90" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J89" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="90" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A90" t="s">
         <v>29</v>
       </c>
@@ -3110,8 +3279,11 @@
       <c r="I90" s="4">
         <v>-3.4041242999999999</v>
       </c>
-    </row>
-    <row r="91" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J90" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="91" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A91" t="s">
         <v>29</v>
       </c>
@@ -3139,8 +3311,11 @@
       <c r="I91" s="4">
         <v>-3.4041242999999999</v>
       </c>
-    </row>
-    <row r="92" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J91" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="92" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A92" t="s">
         <v>29</v>
       </c>
@@ -3169,7 +3344,7 @@
         <v>-3.4057582000000002</v>
       </c>
     </row>
-    <row r="93" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A93" t="s">
         <v>29</v>
       </c>
@@ -3198,7 +3373,7 @@
         <v>-3.4057582000000002</v>
       </c>
     </row>
-    <row r="94" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A94" t="s">
         <v>29</v>
       </c>
@@ -3227,7 +3402,7 @@
         <v>-3.4057582000000002</v>
       </c>
     </row>
-    <row r="95" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A95" t="s">
         <v>29</v>
       </c>
@@ -3255,8 +3430,11 @@
       <c r="I95" s="4">
         <v>-3.4063479999999999</v>
       </c>
-    </row>
-    <row r="96" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J95" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="96" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A96" t="s">
         <v>29</v>
       </c>
@@ -3284,8 +3462,11 @@
       <c r="I96" s="4">
         <v>-3.4063479999999999</v>
       </c>
-    </row>
-    <row r="97" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J96" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="97" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A97" t="s">
         <v>29</v>
       </c>
@@ -3313,8 +3494,11 @@
       <c r="I97" s="4">
         <v>-3.4063479999999999</v>
       </c>
-    </row>
-    <row r="98" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J97" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="98" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A98" t="s">
         <v>29</v>
       </c>
@@ -3342,8 +3526,11 @@
       <c r="I98" s="4">
         <v>-3.4052527000000001</v>
       </c>
-    </row>
-    <row r="99" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J98" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="99" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A99" t="s">
         <v>29</v>
       </c>
@@ -3371,8 +3558,11 @@
       <c r="I99" s="4">
         <v>-3.4052527000000001</v>
       </c>
-    </row>
-    <row r="100" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J99" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="100" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A100" t="s">
         <v>29</v>
       </c>
@@ -3400,8 +3590,11 @@
       <c r="I100" s="4">
         <v>-3.4052527000000001</v>
       </c>
-    </row>
-    <row r="101" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J100" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="101" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A101" t="s">
         <v>29</v>
       </c>
@@ -3430,7 +3623,7 @@
         <v>-3.4041681000000001</v>
       </c>
     </row>
-    <row r="102" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A102" t="s">
         <v>29</v>
       </c>
@@ -3459,7 +3652,7 @@
         <v>-3.4041681000000001</v>
       </c>
     </row>
-    <row r="103" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A103" t="s">
         <v>29</v>
       </c>
@@ -3488,7 +3681,7 @@
         <v>-3.4041681000000001</v>
       </c>
     </row>
-    <row r="104" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A104" t="s">
         <v>29</v>
       </c>
@@ -3516,8 +3709,11 @@
       <c r="I104" s="4">
         <v>-3.4036138</v>
       </c>
-    </row>
-    <row r="105" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J104" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="105" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A105" t="s">
         <v>29</v>
       </c>
@@ -3545,8 +3741,11 @@
       <c r="I105" s="4">
         <v>-3.4036138</v>
       </c>
-    </row>
-    <row r="106" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J105" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="106" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A106" t="s">
         <v>29</v>
       </c>
@@ -3574,8 +3773,11 @@
       <c r="I106" s="4">
         <v>-3.4036138</v>
       </c>
-    </row>
-    <row r="107" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J106" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="107" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A107" t="s">
         <v>29</v>
       </c>
@@ -3603,8 +3805,11 @@
       <c r="I107" s="4">
         <v>-3.4058609</v>
       </c>
-    </row>
-    <row r="108" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J107" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="108" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A108" t="s">
         <v>29</v>
       </c>
@@ -3632,8 +3837,11 @@
       <c r="I108" s="4">
         <v>-3.4058609</v>
       </c>
-    </row>
-    <row r="109" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J108" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="109" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A109" t="s">
         <v>29</v>
       </c>
@@ -3661,8 +3869,11 @@
       <c r="I109" s="4">
         <v>-3.4058609</v>
       </c>
-    </row>
-    <row r="110" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J109" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="110" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A110" t="s">
         <v>29</v>
       </c>
@@ -3690,8 +3901,11 @@
       <c r="I110" s="4">
         <v>-3.4036038</v>
       </c>
-    </row>
-    <row r="111" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J110" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="111" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A111" t="s">
         <v>29</v>
       </c>
@@ -3719,8 +3933,11 @@
       <c r="I111" s="4">
         <v>-3.4036038</v>
       </c>
-    </row>
-    <row r="112" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J111" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="112" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A112" t="s">
         <v>29</v>
       </c>
@@ -3748,8 +3965,11 @@
       <c r="I112" s="4">
         <v>-3.4036038</v>
       </c>
-    </row>
-    <row r="113" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J112" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="113" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A113" t="s">
         <v>29</v>
       </c>
@@ -3777,8 +3997,11 @@
       <c r="I113" s="4">
         <v>-3.4046557000000002</v>
       </c>
-    </row>
-    <row r="114" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J113" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="114" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A114" t="s">
         <v>29</v>
       </c>
@@ -3806,8 +4029,11 @@
       <c r="I114" s="4">
         <v>-3.4046557000000002</v>
       </c>
-    </row>
-    <row r="115" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J114" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="115" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A115" t="s">
         <v>29</v>
       </c>
@@ -3835,8 +4061,11 @@
       <c r="I115" s="4">
         <v>-3.4046557000000002</v>
       </c>
-    </row>
-    <row r="116" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J115" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="116" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A116" t="s">
         <v>29</v>
       </c>
@@ -3864,8 +4093,11 @@
       <c r="I116" s="4">
         <v>-3.4037117000000001</v>
       </c>
-    </row>
-    <row r="117" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J116" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="117" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A117" t="s">
         <v>29</v>
       </c>
@@ -3893,8 +4125,11 @@
       <c r="I117" s="4">
         <v>-3.4037117000000001</v>
       </c>
-    </row>
-    <row r="118" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J117" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="118" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A118" t="s">
         <v>29</v>
       </c>
@@ -3922,8 +4157,11 @@
       <c r="I118" s="4">
         <v>-3.4037117000000001</v>
       </c>
-    </row>
-    <row r="119" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J118" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="119" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A119" t="s">
         <v>29</v>
       </c>
@@ -3951,8 +4189,11 @@
       <c r="I119" s="4">
         <v>-3.4041983999999998</v>
       </c>
-    </row>
-    <row r="120" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J119" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="120" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A120" t="s">
         <v>29</v>
       </c>
@@ -3980,8 +4221,11 @@
       <c r="I120" s="4">
         <v>-3.4041983999999998</v>
       </c>
-    </row>
-    <row r="121" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="J120" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="121" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A121" t="s">
         <v>29</v>
       </c>
@@ -4008,6 +4252,160 @@
       </c>
       <c r="I121" s="4">
         <v>-3.4041983999999998</v>
+      </c>
+      <c r="J121" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="122" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A122" t="s">
+        <v>39</v>
+      </c>
+      <c r="B122" t="s">
+        <v>30</v>
+      </c>
+      <c r="D122" t="s">
+        <v>23</v>
+      </c>
+      <c r="H122" s="4">
+        <v>55.85445</v>
+      </c>
+      <c r="I122" s="4">
+        <v>-3.3304740000000002</v>
+      </c>
+      <c r="J122" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="123" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A123" t="s">
+        <v>39</v>
+      </c>
+      <c r="B123" t="s">
+        <v>30</v>
+      </c>
+      <c r="D123" t="s">
+        <v>10</v>
+      </c>
+      <c r="H123" s="4">
+        <v>55.853965000000002</v>
+      </c>
+      <c r="I123" s="4">
+        <v>-3.3331650000000002</v>
+      </c>
+      <c r="J123" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="124" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A124" t="s">
+        <v>39</v>
+      </c>
+      <c r="B124" t="s">
+        <v>30</v>
+      </c>
+      <c r="D124" t="s">
+        <v>16</v>
+      </c>
+      <c r="H124" s="4">
+        <v>55.852347000000002</v>
+      </c>
+      <c r="I124" s="4">
+        <v>-3.3325879999999999</v>
+      </c>
+      <c r="J124" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="125" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A125" t="s">
+        <v>39</v>
+      </c>
+      <c r="B125" t="s">
+        <v>30</v>
+      </c>
+      <c r="D125" t="s">
+        <v>21</v>
+      </c>
+      <c r="H125" s="4">
+        <v>55.85286</v>
+      </c>
+      <c r="I125" s="4">
+        <v>-3.3298009999999998</v>
+      </c>
+      <c r="J125" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="126" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A126" t="s">
+        <v>39</v>
+      </c>
+      <c r="B126" t="s">
+        <v>8</v>
+      </c>
+      <c r="D126" t="s">
+        <v>17</v>
+      </c>
+      <c r="H126" s="4">
+        <v>55.852832999999997</v>
+      </c>
+      <c r="I126" s="4">
+        <v>-3.3190360000000001</v>
+      </c>
+      <c r="J126" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="127" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A127" t="s">
+        <v>39</v>
+      </c>
+      <c r="B127" t="s">
+        <v>8</v>
+      </c>
+      <c r="D127" t="s">
+        <v>20</v>
+      </c>
+      <c r="H127" s="4">
+        <v>55.851108000000004</v>
+      </c>
+      <c r="I127" s="4">
+        <v>-3.31894</v>
+      </c>
+    </row>
+    <row r="128" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A128" t="s">
+        <v>39</v>
+      </c>
+      <c r="B128" t="s">
+        <v>8</v>
+      </c>
+      <c r="D128" t="s">
+        <v>12</v>
+      </c>
+      <c r="H128" s="4">
+        <v>55.849463999999998</v>
+      </c>
+      <c r="I128" s="4">
+        <v>-3.3190840000000001</v>
+      </c>
+    </row>
+    <row r="129" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A129" t="s">
+        <v>39</v>
+      </c>
+      <c r="B129" t="s">
+        <v>8</v>
+      </c>
+      <c r="D129" t="s">
+        <v>18</v>
+      </c>
+      <c r="H129" s="4">
+        <v>55.849058999999997</v>
+      </c>
+      <c r="I129" s="4">
+        <v>-3.3166329999999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>